<commit_message>
new rule logic and data
</commit_message>
<xml_diff>
--- a/rules/CORE-000892/positive/01/data/unit-test-coreid-FB4301_positive.xlsx
+++ b/rules/CORE-000892/positive/01/data/unit-test-coreid-FB4301_positive.xlsx
@@ -953,6 +953,11 @@
           <t>SCREENING</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2013-03</t>
+        </is>
+      </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
           <t>BEFORE</t>
@@ -993,6 +998,11 @@
           <t>SCREENING</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2013-02</t>
+        </is>
+      </c>
       <c r="I7" s="8" t="inlineStr">
         <is>
           <t>VISIT 0</t>
@@ -1040,6 +1050,11 @@
           <t>2012-03</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>AFTER</t>
+        </is>
+      </c>
       <c r="K8" s="8" t="inlineStr">
         <is>
           <t>AFTER</t>
@@ -1119,6 +1134,11 @@
           <t>SCREENING</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>DURING</t>
+        </is>
+      </c>
       <c r="I10" s="7" t="inlineStr">
         <is>
           <t>VISIT1</t>
@@ -1166,6 +1186,11 @@
           <t>2013-01-11</t>
         </is>
       </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>VISIT99</t>
+        </is>
+      </c>
       <c r="J11" s="11" t="n"/>
       <c r="L11" s="7" t="inlineStr">
         <is>
@@ -1210,7 +1235,11 @@
           <t>BEFORE</t>
         </is>
       </c>
-      <c r="I12" s="9" t="n"/>
+      <c r="I12" s="9" t="inlineStr">
+        <is>
+          <t>VISIT99</t>
+        </is>
+      </c>
       <c r="J12" s="9" t="n"/>
       <c r="L12" s="7" t="inlineStr">
         <is>

</xml_diff>